<commit_message>
Remaster equipment and skills onto the v2.1 Health band.
Scale Armour/Magic Armour to the workbook loadout budgets, grant Grey
defence actions, retune restore/Fortify/Ward, add four plumage sets plus
Focus Ward Orbs and new accessories, and switch Health and Attack Power
on so the new pools match incoming damage.

Co-authored-by: jacobbeebe007-ui <jacobbeebe007-ui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Avian_Ascent_Current_Master_v2.1.xlsx
+++ b/Avian_Ascent_Current_Master_v2.1.xlsx
@@ -58,6 +58,7 @@
     <sheet name="Scaling Model" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="Progression Rules" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="Bird &amp; Classes" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="Equipment Remaster" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +68,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +79,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -115,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -129,6 +134,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -553,7 +559,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>v2.1 locked rules; Attack Power / Health are next-foundation (runtime still weapon-first + Vitality×3).</t>
+          <t>v2.1 Health and Attack Power are live with the equipment remaster.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -563,7 +569,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>LOCKED</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -773,7 +779,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Replace Attack Power and Health formulas, then clear ordinary cooldowns and retune skill numbers.</t>
+          <t>Ordinary cooldown wipe and 52-bird identity pass. Next telemetry ≥200 runs/matchup.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -784,6 +790,34 @@
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>REQUIRED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Equipment remaster</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Worn pools Grey 20/28/36 … Orange 50/70/88. Grey defence actions. 407 items (+4 sets, Focus Ward Orb, new accessories).</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Equipment Rework</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -79848,6 +79882,276 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>V2.1 EQUIPMENT &amp; SKILL REMASTER</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Worn loadout protection (no shield)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Grey</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D3" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" t="n">
+        <v>41</v>
+      </c>
+      <c r="D5" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>35</v>
+      </c>
+      <c r="C6" t="n">
+        <v>49</v>
+      </c>
+      <c r="D6" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>59</v>
+      </c>
+      <c r="D7" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="n">
+        <v>70</v>
+      </c>
+      <c r="D8" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Slot share</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumage 70%</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Headgear 20%</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Anklets 10% + Shield extra 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Restore (2 AP)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>8–14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>≤35% of one 3 AP hit</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Grey from plumage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fortify / Ward (4 AP)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>16–30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>≤75% of one enemy turn</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Grey from Shield / Orb</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>New sets</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tempestweave, Maris Tideplate, Solis Mail, Aeris Silk</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>New off-hand</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Focus Ward Orb (Ward from Grey)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>New accessories</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Stoneband / Galeband anklets, Warden Torque, Aspect Charm</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Catalogue</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>407 items, 141 skills, 48 families</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix remaster verifies and keep rider text aligned with Health-band amounts.
Make the remaster script idempotent, sync Fortify/Ward specials and
bastion rider text, and update combat scenarios plus workbook L1 Health
so the full CI suite passes on the v2.1 pools.

Co-authored-by: jacobbeebe007-ui <jacobbeebe007-ui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Avian_Ascent_Current_Master_v2.1.xlsx
+++ b/Avian_Ascent_Current_Master_v2.1.xlsx
@@ -793,12 +793,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -21496,7 +21490,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Runtime still uses these v1.6 conversions (Vitality × 3, weapon-first 2.5%). Adopted next-foundation rules are on V2 Core Rules, AP Expectation Tests, Hybrid Damage, Affinity and Ultimate Meter.</t>
+          <t>Runtime still uses these v1.6 conversions (5 × Vitality, weapon-first 2.5%). Adopted next-foundation rules are on V2 Core Rules, AP Expectation Tests, Hybrid Damage, Affinity and Ultimate Meter.</t>
         </is>
       </c>
     </row>
@@ -21572,7 +21566,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Each +1 Vitality increases Max Health by 3 (flat).</t>
+          <t>Each +1 Vitality increases Max Health by 5 (flat).</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -21592,7 +21586,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>L1 Max Health = Base Health + Vitality × 3. Later levels add ½ original Base Health before Vitality.</t>
+          <t>L1 Max Health = Size Base + 5 × Vitality + 5 × (Level − 1). Later levels add ½ original Base Health before Vitality.</t>
         </is>
       </c>
     </row>
@@ -22693,7 +22687,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Base Health + Vitality × 3</t>
+          <t>Size Base + 5 × Vitality + 5 × (Level − 1)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -23739,10 +23733,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE5" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="AE5" s="2" t="n">
+        <v>143</v>
       </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
@@ -23921,10 +23913,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE6" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="AE6" s="2" t="n">
+        <v>125</v>
       </c>
       <c r="AF6" s="2" t="inlineStr">
         <is>
@@ -24103,10 +24093,8 @@
           <t>The first Magic weapon skill you use each turn deals 10% additional damage to Magic Armour only. This bonus does not increase Health damage.</t>
         </is>
       </c>
-      <c r="AE7" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="AE7" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="AF7" s="2" t="inlineStr">
         <is>
@@ -24281,10 +24269,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE8" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="AE8" s="2" t="n">
+        <v>154</v>
       </c>
       <c r="AF8" s="2" t="inlineStr">
         <is>
@@ -24459,10 +24445,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE9" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="AE9" s="2" t="n">
+        <v>136</v>
       </c>
       <c r="AF9" s="2" t="inlineStr">
         <is>
@@ -24641,10 +24625,8 @@
           <t>The first Magic weapon skill you use each turn deals 10% additional damage to Magic Armour only. This bonus does not increase Health damage.</t>
         </is>
       </c>
-      <c r="AE10" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="AE10" s="2" t="n">
+        <v>154</v>
       </c>
       <c r="AF10" s="2" t="inlineStr">
         <is>
@@ -24819,10 +24801,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE11" s="2" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="AE11" s="2" t="n">
+        <v>169</v>
       </c>
       <c r="AF11" s="2" t="inlineStr">
         <is>
@@ -25001,10 +24981,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE12" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE12" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF12" s="2" t="inlineStr">
         <is>
@@ -25179,10 +25157,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE13" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="AE13" s="2" t="n">
+        <v>156</v>
       </c>
       <c r="AF13" s="2" t="inlineStr">
         <is>
@@ -25357,10 +25333,8 @@
           <t>Once per turn after you break Magic Armour, the next ailment or stat debuff you apply to that target gains +10 percentage points application chance and lasts 1 additional turn.</t>
         </is>
       </c>
-      <c r="AE14" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="AE14" s="2" t="n">
+        <v>141</v>
       </c>
       <c r="AF14" s="2" t="inlineStr">
         <is>
@@ -25535,10 +25509,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE15" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="AE15" s="2" t="n">
+        <v>159</v>
       </c>
       <c r="AF15" s="2" t="inlineStr">
         <is>
@@ -25713,10 +25685,8 @@
           <t>Once per turn after you break Magic Armour, the next ailment or stat debuff you apply to that target gains +10 percentage points application chance and lasts 1 additional turn.</t>
         </is>
       </c>
-      <c r="AE16" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="AE16" s="2" t="n">
+        <v>149</v>
       </c>
       <c r="AF16" s="2" t="inlineStr">
         <is>
@@ -25891,10 +25861,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE17" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
+      <c r="AE17" s="2" t="n">
+        <v>146</v>
       </c>
       <c r="AF17" s="2" t="inlineStr">
         <is>
@@ -26069,10 +26037,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE18" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="AE18" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="AF18" s="2" t="inlineStr">
         <is>
@@ -26247,10 +26213,8 @@
           <t>Once per turn after you break Magic Armour, the next ailment or stat debuff you apply to that target gains +10 percentage points application chance and lasts 1 additional turn.</t>
         </is>
       </c>
-      <c r="AE19" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="AE19" s="2" t="n">
+        <v>141</v>
       </c>
       <c r="AF19" s="2" t="inlineStr">
         <is>
@@ -26425,10 +26389,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE20" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE20" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF20" s="2" t="inlineStr">
         <is>
@@ -26603,10 +26565,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE21" s="2" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="AE21" s="2" t="n">
+        <v>172</v>
       </c>
       <c r="AF21" s="2" t="inlineStr">
         <is>
@@ -26781,10 +26741,8 @@
           <t>Once per turn after you break Magic Armour, the next ailment or stat debuff you apply to that target gains +10 percentage points application chance and lasts 1 additional turn.</t>
         </is>
       </c>
-      <c r="AE22" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="AE22" s="2" t="n">
+        <v>144</v>
       </c>
       <c r="AF22" s="2" t="inlineStr">
         <is>
@@ -26959,10 +26917,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE23" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="AE23" s="2" t="n">
+        <v>154</v>
       </c>
       <c r="AF23" s="2" t="inlineStr">
         <is>
@@ -27137,10 +27093,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE24" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="AE24" s="2" t="n">
+        <v>177</v>
       </c>
       <c r="AF24" s="2" t="inlineStr">
         <is>
@@ -27315,10 +27269,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE25" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE25" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF25" s="2" t="inlineStr">
         <is>
@@ -27493,10 +27445,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE26" s="2" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="AE26" s="2" t="n">
+        <v>172</v>
       </c>
       <c r="AF26" s="2" t="inlineStr">
         <is>
@@ -27671,10 +27621,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE27" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="AE27" s="2" t="n">
+        <v>177</v>
       </c>
       <c r="AF27" s="2" t="inlineStr">
         <is>
@@ -27853,10 +27801,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE28" s="2" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="AE28" s="2" t="n">
+        <v>162</v>
       </c>
       <c r="AF28" s="2" t="inlineStr">
         <is>
@@ -28031,10 +27977,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE29" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="AE29" s="2" t="n">
+        <v>159</v>
       </c>
       <c r="AF29" s="2" t="inlineStr">
         <is>
@@ -28209,10 +28153,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE30" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="AE30" s="2" t="n">
+        <v>185</v>
       </c>
       <c r="AF30" s="2" t="inlineStr">
         <is>
@@ -28387,10 +28329,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE31" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="AE31" s="2" t="n">
+        <v>165</v>
       </c>
       <c r="AF31" s="2" t="inlineStr">
         <is>
@@ -28569,10 +28509,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE32" s="2" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
+      <c r="AE32" s="2" t="n">
+        <v>170</v>
       </c>
       <c r="AF32" s="2" t="inlineStr">
         <is>
@@ -28747,10 +28685,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE33" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="AE33" s="2" t="n">
+        <v>165</v>
       </c>
       <c r="AF33" s="2" t="inlineStr">
         <is>
@@ -28925,10 +28861,8 @@
           <t>After defeating an enemy, restore 25% of normal Maximum Armour and Magic Armour and gain +5% all damage for the remainder of combat.</t>
         </is>
       </c>
-      <c r="AE34" s="2" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="AE34" s="2" t="n">
+        <v>175</v>
       </c>
       <c r="AF34" s="2" t="inlineStr">
         <is>
@@ -29107,10 +29041,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE35" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="AE35" s="2" t="n">
+        <v>130</v>
       </c>
       <c r="AF35" s="2" t="inlineStr">
         <is>
@@ -29289,10 +29221,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE36" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="AE36" s="2" t="n">
+        <v>135</v>
       </c>
       <c r="AF36" s="2" t="inlineStr">
         <is>
@@ -29467,10 +29397,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE37" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="AE37" s="2" t="n">
+        <v>130</v>
       </c>
       <c r="AF37" s="2" t="inlineStr">
         <is>
@@ -29649,10 +29577,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE38" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="AE38" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="AF38" s="2" t="inlineStr">
         <is>
@@ -29827,10 +29753,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE39" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE39" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF39" s="2" t="inlineStr">
         <is>
@@ -30005,10 +29929,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE40" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="AE40" s="2" t="n">
+        <v>148</v>
       </c>
       <c r="AF40" s="2" t="inlineStr">
         <is>
@@ -30183,10 +30105,8 @@
           <t>The first Magic weapon skill you use each turn deals 10% additional damage to Magic Armour only. This bonus does not increase Health damage.</t>
         </is>
       </c>
-      <c r="AE41" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="AE41" s="2" t="n">
+        <v>133</v>
       </c>
       <c r="AF41" s="2" t="inlineStr">
         <is>
@@ -30361,10 +30281,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE42" s="2" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="AE42" s="2" t="n">
+        <v>164</v>
       </c>
       <c r="AF42" s="2" t="inlineStr">
         <is>
@@ -30539,10 +30457,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE43" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="AE43" s="2" t="n">
+        <v>159</v>
       </c>
       <c r="AF43" s="2" t="inlineStr">
         <is>
@@ -30717,10 +30633,8 @@
           <t>The first Magic weapon skill you use each turn deals 10% additional damage to Magic Armour only. This bonus does not increase Health damage.</t>
         </is>
       </c>
-      <c r="AE44" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="AE44" s="2" t="n">
+        <v>141</v>
       </c>
       <c r="AF44" s="2" t="inlineStr">
         <is>
@@ -30899,10 +30813,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE45" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="AE45" s="2" t="n">
+        <v>177</v>
       </c>
       <c r="AF45" s="2" t="inlineStr">
         <is>
@@ -31077,10 +30989,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE46" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="AE46" s="2" t="n">
+        <v>149</v>
       </c>
       <c r="AF46" s="2" t="inlineStr">
         <is>
@@ -31255,10 +31165,8 @@
           <t>Once per turn after Armour absorbs physical damage, your next Strength weapon skill gains +10 Skill Power.</t>
         </is>
       </c>
-      <c r="AE47" s="2" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
+      <c r="AE47" s="2" t="n">
+        <v>182</v>
       </c>
       <c r="AF47" s="2" t="inlineStr">
         <is>
@@ -31437,10 +31345,8 @@
           <t>Once per turn after a damaging skill hits an ailmented, debuffed or Marked target, restore 2 to the lower of Armour or Magic Armour, capped at its normal maximum. If both pools are full, heal 5% Maximum Health.</t>
         </is>
       </c>
-      <c r="AE48" s="2" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="AE48" s="2" t="n">
+        <v>172</v>
       </c>
       <c r="AF48" s="2" t="inlineStr">
         <is>
@@ -31615,10 +31521,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE49" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE49" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF49" s="2" t="inlineStr">
         <is>
@@ -31793,10 +31697,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE50" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="AE50" s="2" t="n">
+        <v>156</v>
       </c>
       <c r="AF50" s="2" t="inlineStr">
         <is>
@@ -31971,10 +31873,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE51" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="AE51" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="AF51" s="2" t="inlineStr">
         <is>
@@ -32149,10 +32049,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE52" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="AE52" s="2" t="n">
+        <v>151</v>
       </c>
       <c r="AF52" s="2" t="inlineStr">
         <is>
@@ -32327,10 +32225,8 @@
           <t>Once per turn, when you alternate Martial and Magic damaging skills, the second skill restores 2 to the lower protection pool. If both pools are full, it gains +10 Skill Power instead.</t>
         </is>
       </c>
-      <c r="AE53" s="2" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="AE53" s="2" t="n">
+        <v>164</v>
       </c>
       <c r="AF53" s="2" t="inlineStr">
         <is>
@@ -32509,10 +32405,8 @@
           <t>Once per turn, after using Armour Restoration or Fortify, gain Minor Guard Up (+4 Guard) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE54" s="2" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="AE54" s="2" t="n">
+        <v>172</v>
       </c>
       <c r="AF54" s="2" t="inlineStr">
         <is>
@@ -32691,10 +32585,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE55" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="AE55" s="2" t="n">
+        <v>135</v>
       </c>
       <c r="AF55" s="2" t="inlineStr">
         <is>
@@ -32869,10 +32761,8 @@
           <t>Once per turn, if acting before the target, your first Weapon Skill 1 gains +10 Precision. If that skill breaks Armour, gain Minor Agility Up (+4 Agility) until the start of your next turn.</t>
         </is>
       </c>
-      <c r="AE56" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="AE56" s="2" t="n">
+        <v>138</v>
       </c>
       <c r="AF56" s="2" t="inlineStr">
         <is>
@@ -79897,9 +79787,6 @@
           <t>V2.1 EQUIPMENT &amp; SKILL REMASTER</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -80019,12 +79906,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -80102,8 +79984,6 @@
           <t>Tempestweave, Maris Tideplate, Solis Mail, Aeris Silk</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -80116,8 +79996,6 @@
           <t>Focus Ward Orb (Ward from Grey)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -80130,8 +80008,6 @@
           <t>Stoneband / Galeband anklets, Warden Torque, Aspect Charm</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -80144,8 +80020,6 @@
           <t>407 items, 141 skills, 48 families</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>